<commit_message>
feat(math): canonical base-only package, unshipped bonus mode removed, PAR regenerated from uploaded artefact
Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/games/future_spinner/library/future_spinner_full_statistics.xlsx
+++ b/games/future_spinner/library/future_spinner_full_statistics.xlsx
@@ -85,31 +85,31 @@
     <t>1.0</t>
   </si>
   <si>
-    <t>1.496</t>
-  </si>
-  <si>
-    <t>5.52</t>
-  </si>
-  <si>
-    <t>10.012</t>
-  </si>
-  <si>
-    <t>87.51</t>
-  </si>
-  <si>
-    <t>85.628</t>
-  </si>
-  <si>
-    <t>58.553</t>
-  </si>
-  <si>
-    <t>102.256</t>
-  </si>
-  <si>
-    <t>1737.678</t>
-  </si>
-  <si>
-    <t>22054.143</t>
+    <t>1.501</t>
+  </si>
+  <si>
+    <t>6.016</t>
+  </si>
+  <si>
+    <t>8.963</t>
+  </si>
+  <si>
+    <t>62.629</t>
+  </si>
+  <si>
+    <t>71.948</t>
+  </si>
+  <si>
+    <t>58.904</t>
+  </si>
+  <si>
+    <t>114.615</t>
+  </si>
+  <si>
+    <t>1703.053</t>
+  </si>
+  <si>
+    <t>46716.72</t>
   </si>
   <si>
     <t>100000.001</t>
@@ -172,13 +172,13 @@
     <t>{'symbol': 'scatter'}</t>
   </si>
   <si>
-    <t>16.096557805889148</t>
+    <t>15.706694151911536</t>
   </si>
   <si>
     <t>6478</t>
   </si>
   <si>
-    <t>95.07297920192711</t>
+    <t>97.57620875615943</t>
   </si>
 </sst>
 </file>
@@ -541,10 +541,10 @@
         <v>3</v>
       </c>
       <c r="B2">
-        <v>1.496</v>
+        <v>1.501</v>
       </c>
       <c r="C2">
-        <v>0.0003270089365256252</v>
+        <v>0.0001405812654839212</v>
       </c>
       <c r="F2" t="s">
         <v>3</v>
@@ -567,10 +567,10 @@
         <v>4</v>
       </c>
       <c r="B3">
-        <v>5.52</v>
+        <v>6.016</v>
       </c>
       <c r="C3">
-        <v>0.1097623389177903</v>
+        <v>0.09915264902707593</v>
       </c>
       <c r="F3" t="s">
         <v>4</v>
@@ -593,10 +593,10 @@
         <v>5</v>
       </c>
       <c r="B4">
-        <v>10.012</v>
+        <v>8.962999999999999</v>
       </c>
       <c r="C4">
-        <v>0.1272137770572964</v>
+        <v>0.1398661705340271</v>
       </c>
       <c r="F4" t="s">
         <v>5</v>
@@ -619,10 +619,10 @@
         <v>6</v>
       </c>
       <c r="B5">
-        <v>87.51000000000001</v>
+        <v>62.629</v>
       </c>
       <c r="C5">
-        <v>0.03864770427424709</v>
+        <v>0.05423291112935776</v>
       </c>
       <c r="F5" t="s">
         <v>6</v>
@@ -645,10 +645,10 @@
         <v>7</v>
       </c>
       <c r="B6">
-        <v>85.628</v>
+        <v>71.94799999999999</v>
       </c>
       <c r="C6">
-        <v>0.08568193573618406</v>
+        <v>0.1009376958760442</v>
       </c>
       <c r="F6" t="s">
         <v>7</v>
@@ -671,10 +671,10 @@
         <v>8</v>
       </c>
       <c r="B7">
-        <v>58.553</v>
+        <v>58.904</v>
       </c>
       <c r="C7">
-        <v>0.2421270111808186</v>
+        <v>0.2364316821474623</v>
       </c>
       <c r="F7" t="s">
         <v>8</v>
@@ -697,10 +697,10 @@
         <v>9</v>
       </c>
       <c r="B8">
-        <v>102.256</v>
+        <v>114.615</v>
       </c>
       <c r="C8">
-        <v>0.2696212688504349</v>
+        <v>0.2442982649334291</v>
       </c>
       <c r="F8" t="s">
         <v>9</v>
@@ -723,10 +723,10 @@
         <v>10</v>
       </c>
       <c r="B9">
-        <v>1737.678</v>
+        <v>1703.053</v>
       </c>
       <c r="C9">
-        <v>0.03509712775707251</v>
+        <v>0.03598196364583187</v>
       </c>
       <c r="F9" t="s">
         <v>10</v>
@@ -749,10 +749,10 @@
         <v>11</v>
       </c>
       <c r="B10">
-        <v>22054.143</v>
+        <v>46716.72</v>
       </c>
       <c r="C10">
-        <v>0.005021827238826386</v>
+        <v>0.002458081389937359</v>
       </c>
       <c r="F10" t="s">
         <v>11</v>
@@ -934,7 +934,7 @@
         <v>100000.001</v>
       </c>
       <c r="C17">
-        <v>0.04999999969878099</v>
+        <v>0.04999999969885738</v>
       </c>
       <c r="F17" t="s">
         <v>19</v>
@@ -997,13 +997,13 @@
         <v>34</v>
       </c>
       <c r="B23">
-        <v>913.17</v>
+        <v>859.47</v>
       </c>
       <c r="C23">
-        <v>392.12</v>
+        <v>360.4</v>
       </c>
       <c r="D23">
-        <v>319.51</v>
+        <v>305.18</v>
       </c>
       <c r="G23" t="s">
         <v>34</v>
@@ -1021,13 +1021,13 @@
         <v>34</v>
       </c>
       <c r="N23">
-        <v>221.3</v>
+        <v>192.1</v>
       </c>
       <c r="O23">
-        <v>78.7</v>
+        <v>72.8</v>
       </c>
       <c r="P23">
-        <v>202.3</v>
+        <v>180.8</v>
       </c>
     </row>
     <row r="24" spans="1:16">
@@ -1035,13 +1035,13 @@
         <v>35</v>
       </c>
       <c r="B24">
-        <v>509.7</v>
+        <v>528.21</v>
       </c>
       <c r="C24">
-        <v>200.16</v>
+        <v>209.76</v>
       </c>
       <c r="D24">
-        <v>128.94</v>
+        <v>139.49</v>
       </c>
       <c r="G24" t="s">
         <v>35</v>
@@ -1059,13 +1059,13 @@
         <v>35</v>
       </c>
       <c r="N24">
-        <v>76.09999999999999</v>
+        <v>77.09999999999999</v>
       </c>
       <c r="O24">
-        <v>109.1</v>
+        <v>102.5</v>
       </c>
       <c r="P24">
-        <v>87.09999999999999</v>
+        <v>89.7</v>
       </c>
     </row>
     <row r="25" spans="1:16">
@@ -1073,13 +1073,13 @@
         <v>36</v>
       </c>
       <c r="B25">
-        <v>113.67</v>
+        <v>112.93</v>
       </c>
       <c r="C25">
-        <v>96.45</v>
+        <v>88.45</v>
       </c>
       <c r="D25">
-        <v>124.91</v>
+        <v>108.92</v>
       </c>
       <c r="G25" t="s">
         <v>36</v>
@@ -1097,13 +1097,13 @@
         <v>36</v>
       </c>
       <c r="N25">
-        <v>95.59999999999999</v>
+        <v>92.90000000000001</v>
       </c>
       <c r="O25">
-        <v>89.8</v>
+        <v>84.8</v>
       </c>
       <c r="P25">
-        <v>124.1</v>
+        <v>112</v>
       </c>
     </row>
     <row r="26" spans="1:16">
@@ -1111,13 +1111,13 @@
         <v>37</v>
       </c>
       <c r="B26">
-        <v>94.12</v>
+        <v>92.28</v>
       </c>
       <c r="C26">
-        <v>61.17</v>
+        <v>62.03</v>
       </c>
       <c r="D26">
-        <v>82.08</v>
+        <v>82.45</v>
       </c>
       <c r="G26" t="s">
         <v>37</v>
@@ -1135,13 +1135,13 @@
         <v>37</v>
       </c>
       <c r="N26">
-        <v>76.5</v>
+        <v>77.5</v>
       </c>
       <c r="O26">
-        <v>89.09999999999999</v>
+        <v>88</v>
       </c>
       <c r="P26">
-        <v>103.7</v>
+        <v>104.4</v>
       </c>
     </row>
     <row r="27" spans="1:16">
@@ -1149,13 +1149,13 @@
         <v>38</v>
       </c>
       <c r="B27">
-        <v>55.04</v>
+        <v>54.07</v>
       </c>
       <c r="C27">
-        <v>46.52</v>
+        <v>41.24</v>
       </c>
       <c r="D27">
-        <v>66.53</v>
+        <v>67.12</v>
       </c>
       <c r="G27" t="s">
         <v>38</v>
@@ -1173,13 +1173,13 @@
         <v>38</v>
       </c>
       <c r="N27">
-        <v>103.3</v>
+        <v>103</v>
       </c>
       <c r="O27">
-        <v>71.59999999999999</v>
+        <v>74.40000000000001</v>
       </c>
       <c r="P27">
-        <v>74.3</v>
+        <v>76.5</v>
       </c>
     </row>
     <row r="28" spans="1:16">
@@ -1187,13 +1187,13 @@
         <v>39</v>
       </c>
       <c r="B28">
-        <v>20.98</v>
+        <v>19.69</v>
       </c>
       <c r="C28">
-        <v>21.37</v>
+        <v>22.27</v>
       </c>
       <c r="D28">
-        <v>24.11</v>
+        <v>23.55</v>
       </c>
       <c r="G28" t="s">
         <v>39</v>
@@ -1211,13 +1211,13 @@
         <v>39</v>
       </c>
       <c r="N28">
-        <v>85</v>
+        <v>89.8</v>
       </c>
       <c r="O28">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="P28">
-        <v>96.5</v>
+        <v>95</v>
       </c>
     </row>
     <row r="29" spans="1:16">
@@ -1225,13 +1225,13 @@
         <v>40</v>
       </c>
       <c r="B29">
-        <v>27.63</v>
+        <v>25.4</v>
       </c>
       <c r="C29">
-        <v>42.15</v>
+        <v>35.86</v>
       </c>
       <c r="D29">
-        <v>70.26000000000001</v>
+        <v>73.31</v>
       </c>
       <c r="G29" t="s">
         <v>40</v>
@@ -1249,13 +1249,13 @@
         <v>40</v>
       </c>
       <c r="N29">
-        <v>83.40000000000001</v>
+        <v>85.2</v>
       </c>
       <c r="O29">
-        <v>105.5</v>
+        <v>104.7</v>
       </c>
       <c r="P29">
-        <v>136</v>
+        <v>126.1</v>
       </c>
     </row>
     <row r="30" spans="1:16">
@@ -1263,13 +1263,13 @@
         <v>41</v>
       </c>
       <c r="B30">
-        <v>19.18</v>
+        <v>19.03</v>
       </c>
       <c r="C30">
-        <v>24.58</v>
+        <v>27.16</v>
       </c>
       <c r="D30">
-        <v>64.94</v>
+        <v>65.56</v>
       </c>
       <c r="G30" t="s">
         <v>41</v>
@@ -1287,13 +1287,13 @@
         <v>41</v>
       </c>
       <c r="N30">
-        <v>84.59999999999999</v>
+        <v>83.59999999999999</v>
       </c>
       <c r="O30">
-        <v>101.4</v>
+        <v>104.7</v>
       </c>
       <c r="P30">
-        <v>98</v>
+        <v>96.8</v>
       </c>
     </row>
     <row r="35" spans="1:4">

</xml_diff>